<commit_message>
Added new RDF data schemes and visual schemes for environment-table40-42, and fixed XLSX spreadsheets for environment-table40-42
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/environment-table40.xlsx
+++ b/sources/table_normalization/xlsx/environment-table40.xlsx
@@ -969,9 +969,6 @@
       <c r="A12" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B12" s="6"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
       <c r="E12" s="4">
         <f>AVERAGE(E2:E11)</f>
         <v>51.2</v>
@@ -986,9 +983,6 @@
       <c r="A13" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B13" s="6"/>
-      <c r="C13" s="6"/>
-      <c r="D13" s="6"/>
       <c r="E13" s="4">
         <f>STDEV(E2:E11)</f>
         <v>38.926711765687202</v>
@@ -1003,9 +997,6 @@
       <c r="A14" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="B14" s="6"/>
-      <c r="C14" s="6"/>
-      <c r="D14" s="6"/>
       <c r="E14" s="4">
         <f>E13/SQRT(10)</f>
         <v>12.3097071000446</v>
@@ -1220,9 +1211,6 @@
       <c r="A26" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B26" s="6"/>
-      <c r="C26" s="6"/>
-      <c r="D26" s="6"/>
       <c r="E26" s="4">
         <f>AVERAGE(E16:E25)</f>
         <v>133.1</v>
@@ -1236,9 +1224,6 @@
       <c r="A27" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B27" s="6"/>
-      <c r="C27" s="6"/>
-      <c r="D27" s="6"/>
       <c r="E27" s="4">
         <f>STDEV(E16:E25)</f>
         <v>39.436165015263697</v>
@@ -1252,9 +1237,6 @@
       <c r="A28" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="B28" s="6"/>
-      <c r="C28" s="6"/>
-      <c r="D28" s="6"/>
       <c r="E28" s="4">
         <f>E27/SQRT(10)</f>
         <v>12.4708103630482</v>
@@ -1588,9 +1570,6 @@
       <c r="A46" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B46" s="6"/>
-      <c r="C46" s="6"/>
-      <c r="D46" s="6"/>
       <c r="E46" s="4">
         <f>AVERAGE(E30:E45)</f>
         <v>225.9375</v>
@@ -1604,9 +1583,6 @@
       <c r="A47" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B47" s="6"/>
-      <c r="C47" s="6"/>
-      <c r="D47" s="6"/>
       <c r="E47" s="4">
         <f>STDEV(E30:E45)</f>
         <v>41.771551323837599</v>
@@ -1620,9 +1596,6 @@
       <c r="A48" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="B48" s="6"/>
-      <c r="C48" s="6"/>
-      <c r="D48" s="6"/>
       <c r="E48" s="4">
         <f>E47/SQRT(16)</f>
         <v>10.4428878309594</v>
@@ -1916,9 +1889,6 @@
       <c r="A64" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B64" s="6"/>
-      <c r="C64" s="6"/>
-      <c r="D64" s="6"/>
       <c r="E64" s="4">
         <f>AVERAGE(E50:E63)</f>
         <v>166.71428571428601</v>
@@ -1932,9 +1902,6 @@
       <c r="A65" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B65" s="6"/>
-      <c r="C65" s="6"/>
-      <c r="D65" s="6"/>
       <c r="E65" s="4">
         <f>STDEV(E50:E63)</f>
         <v>70.0674714075694</v>
@@ -1948,9 +1915,6 @@
       <c r="A66" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="B66" s="6"/>
-      <c r="C66" s="6"/>
-      <c r="D66" s="6"/>
       <c r="E66" s="4">
         <f>E65/SQRT(14)</f>
         <v>18.726319426050299</v>
@@ -2124,9 +2088,6 @@
       <c r="A76" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B76" s="6"/>
-      <c r="C76" s="6"/>
-      <c r="D76" s="6"/>
       <c r="E76" s="4">
         <f>AVERAGE(E68:E75)</f>
         <v>258.625</v>
@@ -2140,9 +2101,6 @@
       <c r="A77" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B77" s="6"/>
-      <c r="C77" s="6"/>
-      <c r="D77" s="6"/>
       <c r="E77" s="4">
         <f>STDEV(E68:E75)</f>
         <v>31.441271784528201</v>
@@ -2156,9 +2114,6 @@
       <c r="A78" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="B78" s="6"/>
-      <c r="C78" s="6"/>
-      <c r="D78" s="6"/>
       <c r="E78" s="4">
         <f>E77/SQRT(8)</f>
         <v>11.1161682439846</v>
@@ -2352,9 +2307,6 @@
       <c r="A89" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B89" s="6"/>
-      <c r="C89" s="6"/>
-      <c r="D89" s="6"/>
       <c r="E89" s="4">
         <f>AVERAGE(E80:E88)</f>
         <v>245.222222222222</v>
@@ -2368,9 +2320,6 @@
       <c r="A90" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B90" s="6"/>
-      <c r="C90" s="6"/>
-      <c r="D90" s="6"/>
       <c r="E90" s="4">
         <f>STDEV(E80:E88)</f>
         <v>36.965449333728401</v>
@@ -2384,9 +2333,6 @@
       <c r="A91" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="B91" s="6"/>
-      <c r="C91" s="6"/>
-      <c r="D91" s="6"/>
       <c r="E91" s="4">
         <f>E90/SQRT(9)</f>
         <v>12.3218164445761</v>

</xml_diff>